<commit_message>
feat(metas): metas do Ciclo 14, com Bronze 2 13706 e Bronze 5
Receita, meta de ativos e R$/ativo copiados da planilha do ciclo nos 15
setores existentes. Multimarca, cabelo e make inalterados nesses setores.

Setores novos, com % iguais aos demais Bronzes (73/36/35) e Qtd sobre a
meta de ativos:
- BRONZE 2 / Todas as cidades 13706 (MARILIA): 60.000 / 110 / 550
- BRONZE 5 / CORURIPE / TEOTONIO / (RODRIGO): 30.000 / 82 / 500

Bronze 1 Coruripe volta para a NATALI. As chaves seguem o nome do setor
no export de vendas, nao o da planilha de metas (que chama o Bronze da
Bruna de "BRONZE 1" e o Bronze 5 de "CORURIPE / JUNQUEIRO"); conferido
contra um ConsultaRankingVendas atual: as 18 metas casam com um setor.

MARILIA entra no mapa padrao do Slack.

Bercario Franquia segue com 172 ativos ate chegar a base do Ciclo 14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -330,7 +330,7 @@
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="53.421875" customWidth="1" min="1" max="1"/>
@@ -401,7 +401,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>RODRIGO</t>
+          <t>NATALI</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -410,11 +410,11 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>R$ 400,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -449,7 +449,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>R$ 70.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
@@ -457,7 +457,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>R$ 600,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -492,15 +492,15 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>R$ 600,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 45.000,00</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>R$ 600,00</t>
+          <t>R$ 500,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -578,7 +578,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>R$ 110.000,00</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.000,00</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -621,7 +621,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>R$ 160.000,00</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
@@ -629,7 +629,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.300,00</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>R$ 160.000,00</t>
+          <t>R$ 135.000,00</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>R$ 1.200,00</t>
+          <t>R$ 1.100,00</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -707,15 +707,15 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>R$ 420.000,00</t>
+          <t>R$ 340.000,00</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>R$ 2.200,00</t>
+          <t>R$ 1.900,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>R$ 350.000,00</t>
+          <t>R$ 310.000,00</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>R$ 3.900,00</t>
+          <t>R$ 3.500,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>R$ 750.000,00</t>
+          <t>R$ 1.500.000,00</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>R$ 25.000,00</t>
+          <t>R$ 53.000,00</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -836,7 +836,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 215.000,00</t>
+          <t>R$ 260.000,00</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -844,7 +844,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>R$ 1.900,00</t>
+          <t>R$ 2.500,00</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -879,7 +879,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 80.000,00</t>
+          <t>R$ 60.000,00</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -887,7 +887,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>R$ 650,00</t>
+          <t>R$ 550,00</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 125.000,00</t>
+          <t>R$ 135.000,00</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -965,7 +965,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R$ 120.000,00</t>
+          <t>R$ 130.000,00</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1008,15 +1008,15 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R$ 400.000,00</t>
+          <t>R$ 520.000,00</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>R$ 4.800,00</t>
+          <t>R$ 7.500,00</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1075,6 +1075,92 @@
       </c>
       <c r="K17" s="1" t="n">
         <v>62</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>BRONZE 2 / Todas as Cidades 13706</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>MARILIA</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>R$ 60.000,00</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>R$ 550,00</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G18" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I18" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>BRONZE 5 / CORURIPE / TEOTÔNIO /</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>RODRIGO</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>R$ 30.000,00</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>82</v>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>R$ 500,00</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>